<commit_message>
correccion de errores formatos
correccion de errores al generar los formatos de los movimientos
</commit_message>
<xml_diff>
--- a/backend/static/plantillas/formato-traslado.xlsx
+++ b/backend/static/plantillas/formato-traslado.xlsx
@@ -35,7 +35,7 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Humanst521 BT"/>
+        <rFont val="Arial"/>
         <b/>
         <color theme="1"/>
         <sz val="11.0"/>
@@ -44,7 +44,7 @@
     </r>
     <r>
       <rPr>
-        <rFont val="Humanst521 BT"/>
+        <rFont val="Arial"/>
         <b val="0"/>
         <color rgb="FF969696"/>
         <sz val="11.0"/>
@@ -190,7 +190,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -212,12 +212,6 @@
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
-      <name val="Humanst521 BT"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11.0"/>
-      <color rgb="FFFF0000"/>
       <name val="Humanst521 BT"/>
     </font>
     <font>
@@ -547,7 +541,7 @@
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="9" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -556,10 +550,10 @@
     <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="9" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -571,7 +565,7 @@
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -595,45 +589,45 @@
     <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="12" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="13" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="14" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="15" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="15" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="16" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="16" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="17" fillId="0" fontId="9" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="17" fillId="0" fontId="8" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="18" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="18" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="19" fillId="0" fontId="9" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="19" fillId="0" fontId="8" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="20" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="20" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="21" fillId="0" fontId="9" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="21" fillId="0" fontId="8" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="22" fillId="0" fontId="9" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="22" fillId="0" fontId="8" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="23" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="23" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="24" fillId="0" fontId="9" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="24" fillId="0" fontId="8" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -887,7 +881,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="23.29"/>
-    <col customWidth="1" min="2" max="2" width="26.71"/>
+    <col customWidth="1" min="2" max="2" width="37.14"/>
     <col customWidth="1" min="3" max="3" width="37.86"/>
     <col customWidth="1" min="4" max="4" width="30.71"/>
     <col customWidth="1" min="5" max="26" width="10.0"/>

</xml_diff>